<commit_message>
More updates on PCB design
I forgot to push my changes for the last week, but I layed out the components and began routing traces and copper pours.
</commit_message>
<xml_diff>
--- a/Battery Charger Project/Excel/BOM/BOM V2 UNIT.xlsx
+++ b/Battery Charger Project/Excel/BOM/BOM V2 UNIT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Verrazano\Acedemic\Research\Battery-Charger\Battery Charger Project\Excel\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC5E4F78-10C8-4999-9D5B-6A34B8E08944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{832AC17C-6418-4DD0-AE92-E1B66B961976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{399A400B-C522-4FE4-B704-6D3A9F06170E}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8928" xr2:uid="{399A400B-C522-4FE4-B704-6D3A9F06170E}"/>
   </bookViews>
   <sheets>
     <sheet name="Minimum" sheetId="3" r:id="rId1"/>

</xml_diff>